<commit_message>
feat: faculty assignment with semester selector, auto-save marks with debounce+badge, dynamic semester rollover
</commit_message>
<xml_diff>
--- a/Data/Faculty_Records.xlsx
+++ b/Data/Faculty_Records.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Belal\Antigravity workspace\Data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Belal\Antigravity workspace\CSE-412\EWU-Portal-System-main\EWU-Portal-System-main\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F15CFB5-2F1B-41C4-BF16-F24E6F126701}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2BEC21C7-AECF-437E-85ED-01BAE7739243}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="65">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="33">
   <si>
     <t>Faculty Initial</t>
   </si>
@@ -115,106 +115,10 @@
     <t>Rajshahi, Bangladesh</t>
   </si>
   <si>
-    <t>TJ</t>
-  </si>
-  <si>
-    <t>Dr. Taskeed Jabid</t>
-  </si>
-  <si>
-    <t>belal.60466046.6@gmail.com</t>
-  </si>
-  <si>
-    <t>Gulshan, Dhaka</t>
-  </si>
-  <si>
-    <t>Khulna, Bangladesh</t>
-  </si>
-  <si>
-    <t>Dr. Mohammad Rezwanul Huq</t>
-  </si>
-  <si>
-    <t>belal.60466046.7@gmail.com</t>
-  </si>
-  <si>
-    <t>Uttara, Dhaka</t>
-  </si>
-  <si>
-    <t>Barisal, Bangladesh</t>
-  </si>
-  <si>
-    <t>Dr. Anup Kumar Paul</t>
-  </si>
-  <si>
-    <t>belal.60466046.10@gmail.com</t>
-  </si>
-  <si>
-    <t>Dhanmondi, Dhaka</t>
-  </si>
-  <si>
-    <t>Rangpur, Bangladesh</t>
-  </si>
-  <si>
-    <t>AH</t>
-  </si>
-  <si>
-    <t>Dr. Anisul Haque</t>
-  </si>
-  <si>
-    <t>rootmass77@gmail.com</t>
-  </si>
-  <si>
-    <t>EEE</t>
-  </si>
-  <si>
-    <t>Bashundhara R/A, Dhaka</t>
-  </si>
-  <si>
-    <t>Comilla, Bangladesh</t>
-  </si>
-  <si>
-    <t>KA</t>
-  </si>
-  <si>
-    <t>Dr. Khairul Alam</t>
-  </si>
-  <si>
-    <t>rootmass08@gmail.com</t>
-  </si>
-  <si>
-    <t>Professor &amp; Chairperson</t>
-  </si>
-  <si>
-    <t>Mohammadpur, Dhaka</t>
-  </si>
-  <si>
-    <t>Feni, Bangladesh</t>
-  </si>
-  <si>
     <t>Dr. Mohammad Mojammel Al Hakim</t>
   </si>
   <si>
-    <t>tabassumaroni207@gmail.com</t>
-  </si>
-  <si>
-    <t>Khilgaon, Dhaka</t>
-  </si>
-  <si>
-    <t>Mymensingh, Bangladesh</t>
-  </si>
-  <si>
-    <t>DAKP</t>
-  </si>
-  <si>
     <t>MMAH</t>
-  </si>
-  <si>
-    <t>DMRH</t>
-  </si>
-  <si>
-    <t>Tabassum Aroni</t>
-  </si>
-  <si>
-    <t>TA</t>
   </si>
 </sst>
 </file>
@@ -648,10 +552,10 @@
     </row>
     <row r="2" spans="1:8" ht="15" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>61</v>
+        <v>32</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>56</v>
+        <v>31</v>
       </c>
       <c r="C2" s="3" t="s">
         <v>8</v>
@@ -751,160 +655,64 @@
       </c>
     </row>
     <row r="6" spans="1:8" ht="15" x14ac:dyDescent="0.3">
-      <c r="A6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>33</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="F6" s="3" t="s">
-        <v>34</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>35</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A6" s="2"/>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="2"/>
     </row>
     <row r="7" spans="1:8" ht="15" x14ac:dyDescent="0.3">
-      <c r="A7" s="4" t="s">
-        <v>62</v>
-      </c>
-      <c r="B7" s="5" t="s">
-        <v>36</v>
-      </c>
-      <c r="C7" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>9</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="G7" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="A7" s="4"/>
+      <c r="B7" s="5"/>
+      <c r="C7" s="5"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="5"/>
+      <c r="F7" s="5"/>
+      <c r="G7" s="5"/>
+      <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" ht="15" x14ac:dyDescent="0.3">
-      <c r="A8" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="B8" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D8" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="F8" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A8" s="2"/>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="2"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="2"/>
     </row>
     <row r="9" spans="1:8" ht="15" x14ac:dyDescent="0.3">
-      <c r="A9" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="B9" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C9" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="G9" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="A9" s="4"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="5"/>
+      <c r="F9" s="5"/>
+      <c r="G9" s="5"/>
+      <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" ht="15" x14ac:dyDescent="0.3">
-      <c r="A10" s="2" t="s">
-        <v>50</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="F10" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G10" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="H10" s="2" t="s">
-        <v>13</v>
-      </c>
+      <c r="A10" s="2"/>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+      <c r="D10" s="2"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="2"/>
     </row>
     <row r="11" spans="1:8" ht="15" x14ac:dyDescent="0.3">
-      <c r="A11" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>47</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>17</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>58</v>
-      </c>
-      <c r="G11" s="5" t="s">
-        <v>59</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>13</v>
-      </c>
+      <c r="A11" s="4"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="5"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="5"/>
+      <c r="H11" s="4"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>